<commit_message>
lc excel sheet updated
</commit_message>
<xml_diff>
--- a/75_questions/75 Questions.xlsx
+++ b/75_questions/75 Questions.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shan/Workspace/leet-code-practice/75_questions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63FCBC4B-600F-674D-91DC-D46C5FE57C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35BFB69-6663-DD40-8C55-C5F7D56913AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17140" xr2:uid="{4DA75435-538F-5544-B769-C24FC4EFB658}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{4DA75435-538F-5544-B769-C24FC4EFB658}"/>
   </bookViews>
   <sheets>
     <sheet name="Easy" sheetId="1" r:id="rId1"/>
+    <sheet name="Medium" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="101">
   <si>
     <t>Question</t>
   </si>
@@ -312,9 +313,6 @@
 </t>
   </si>
   <si>
-    <t>Reverse Words of a String</t>
-  </si>
-  <si>
     <t>Given an input string s, reverse the order of the words.
 A word is defined as a sequence of non-space characters. The words in s will be separated by at least one space.
 Return a string of the words in reverse order concatenated by a single space.
@@ -327,12 +325,6 @@
         s.reverse()
         s = " ".join(s)
         return s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Syntax:
-split() : Split the string into a list 
-reverse() : Reverse the sorting order of the elements 
-"".join() : Takes all the items in an iterable and join them into one string </t>
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-words-in-a-string/description/?envType=study-plan-v2&amp;envId=leetcode-75</t>
@@ -356,15 +348,6 @@
                 i += 1
             i += 1
         return nums</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Syntax:
-pop() : Remove by index and returns the value 
-remove() : remove by value
-del : remove by index and does not return the value
-Use pop() if need to access or use the removed value
-Use del if only need to remove the element and do not need the removed value 
-</t>
   </si>
   <si>
     <t>Is Subsequence</t>
@@ -390,9 +373,6 @@
                 i += 1
             j += 1
         return True if i == s1 else False</t>
-  </si>
-  <si>
-    <t>Maximum Average Subarray</t>
   </si>
   <si>
     <t>Sliding window</t>
@@ -466,12 +446,429 @@
   <si>
     <t>https://leetcode.com/problems/find-pivot-index/?envType=study-plan-v2&amp;envId=leetcode-75</t>
   </si>
+  <si>
+    <t>Find the Difference of the Two Arrays</t>
+  </si>
+  <si>
+    <t>Array + Hash Table</t>
+  </si>
+  <si>
+    <t>Given two 0-indexed integer arrays nums1 and nums2, return a list answer of size 2 where:
+- answer[0] is a list of all distinct integers in nums1 which are not present in nums2.
+- answer[1] is a list of all distinct integers in nums2 which are not present in nums1.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def findDifference(self, nums1: list[int], nums2: list[int]) -&gt; list[list[int]]:
+        nums1 = set(nums1)
+        nums2 = set(nums2)
+        not_in_2 = nums1 - nums2
+        not_in_1 = nums2 - nums1
+        return [list(not_in_2), list(not_in_1)]</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def findDifference(self, nums1: list[int], nums2: list[int]) -&gt; list[list[int]]:
+        not_in_1 = set()
+        not_in_2 = set()
+        for i in nums1:
+            if i not in nums2:
+                not_in_2.add(i)
+        for j in nums2:
+            if j not in nums1:
+                not_in_1.add(j)
+        not_in_2_list = list(not_in_2)
+        not_in_1_list = list(not_in_1)
+        return [not_in_2_list, not_in_1_list]</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def findDifference(self, nums1: list[int], nums2: list[int]) -&gt; list[list[int]]:
+        nums1 = set(nums1)
+        nums2 = set(nums2)
+        distinct_in_nums1 = nums1.difference(nums2)
+        distinct_in_nums2 = nums2.difference(nums1)
+        return [list(distinct_in_nums1), list(distinct_in_nums2)]</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-the-difference-of-two-arrays/?envType=study-plan-v2&amp;envId=leetcode-75</t>
+  </si>
+  <si>
+    <t>Unique Number of Occurrences</t>
+  </si>
+  <si>
+    <t>Given an array of integers arr, return true if the number of occurrences of each value in the array is unique or false otherwise.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def uniqueOccurrences(self, arr: list[int]) -&gt; bool:
+        counts = Counter(arr)
+        unique_counts = set(counts.values())
+        if len(counts) == len(unique_counts):
+            return True
+        return False</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Syntax:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>split()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : Split the string into a list 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>reverse()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : Reverse the sorting order of the elements 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"".join() </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Takes all the items in an iterable and join them into one string </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Syntax:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>pop()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : Remove by index and returns the value 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>remove()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : remove by value
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>del :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> remove by index and does not return the value
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">Use pop() if need to access or use the removed value
+Use del if only need to remove the element and do not need the removed value 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Python set difference : 
+set1 = {...}
+set2 = {...}
+return the set that contains the items that only exist in set1 and not in set2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>newSet = set1.difference(set2)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+newSet = set1 - set2</t>
+    </r>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/unique-number-of-occurrences/?envType=study-plan-v2&amp;envId=leetcode-75</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Syntax:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>Counter()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : Count frequency of elements in an iterable </t>
+    </r>
+  </si>
+  <si>
+    <t>Maximum Average Subarray I</t>
+  </si>
+  <si>
+    <t>Reverse Words in a String</t>
+  </si>
+  <si>
+    <t>Container With Most Water</t>
+  </si>
+  <si>
+    <t>Array + Two pointers + Greedy</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/container-with-most-water/description/?envType=study-plan-v2&amp;envId=leetcode-75</t>
+  </si>
+  <si>
+    <t>You are given an integer array height of length n. There are n vertical lines drawn such that the two endpoints of the ith line are (i, 0) and (i, height[i]).
+Find two lines that together with the x-axis form a container, such that the container contains the most water.
+Return the maximum amount of water a container can store.
+Notice that you may not slant the container.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def maxArea(self, height: List[int]) -&gt; int:
+        left = 0
+        right = len(height) - 1
+        res = 0
+        while left &lt; right:
+            area = (right - left) * min(height[left], height[right])
+            res = max(res, area)
+            if height[left] &lt; height[right]:
+                left += 1
+            else:
+                right -= 1
+        return res</t>
+  </si>
+  <si>
+    <t>Max Number of K-Sum Pairs</t>
+  </si>
+  <si>
+    <t>Array + Hash Table + Two pointers + Sorting</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/max-number-of-k-sum-pairs/description/?envType=study-plan-v2&amp;envId=leetcode-75</t>
+  </si>
+  <si>
+    <t>You are given an integer array nums and an integer k.
+In one operation, you can pick two numbers from the array whose sum equals k and remove them from the array.
+Return the maximum number of operations you can perform on the array.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class Solution:
+    def maxOperations(self, nums: List[int], k: int) -&gt; int:
+        nums = sorted(nums)
+        total_ops = 0
+        left = 0
+        right = len(nums) - 1
+        while left &lt; right:
+            if nums[left] + nums[right] == k:
+                total_ops += 1
+                left +=1
+                right -= 1
+            elif nums[left] + nums[right] &gt; k:
+                right -= 1
+            else:
+                left += 1
+        return total_ops
+                </t>
+  </si>
+  <si>
+    <t>Maximum Depth of Binary Tree</t>
+  </si>
+  <si>
+    <t>DFS + BFS + Binary Tree</t>
+  </si>
+  <si>
+    <t>Given the root of a binary tree, return its maximum depth.
+A binary tree's maximum depth is the number of nodes along the longest path from the root node down to the farthest leaf node.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def maxDepth(self, root: Optional[TreeNode]) -&gt; int:
+        # Iterative DFS solution
+        if not root:
+            return 0
+        stack = []
+        stack.append([root, 1])
+        res = 1
+        while stack:
+            node, depth = stack.pop()
+            if node:
+                res = max(res, depth)
+                stack.append([node.left, depth + 1])
+                stack.append([node.right, depth + 1])
+        return res</t>
+  </si>
+  <si>
+    <t>Leaf-Similar Trees</t>
+  </si>
+  <si>
+    <t>Tree + DFS + Binary Tree</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/description/?envType=study-plan-v2&amp;envId=leetcode-75</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/leaf-similar-trees/description/?envType=study-plan-v2&amp;envId=leetcode-75</t>
+  </si>
+  <si>
+    <t>Product of Array Except Self</t>
+  </si>
+  <si>
+    <t>Array + Prefix Sum</t>
+  </si>
+  <si>
+    <t>Given an integer array nums, return an array answer such that answer[i] is equal to the product of all the elements of nums except nums[i].
+The product of any prefix or suffix of nums is guaranteed to fit in a 32-bit integer.
+You must write an algorithm that runs in O(n) time and without using the division operation.</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/product-of-array-except-self/description/?envType=study-plan-v2&amp;envId=leetcode-75</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def productExceptSelf(self, nums: List[int]) -&gt; List[int]:
+        res = [1] * len(nums)
+        prefix = 1
+        for i in range(len(nums)):
+            res[i] = prefix
+            prefix *= nums[i]
+        postfix = 1
+        for i in reversed(range(len(nums))):
+            res[i] *= postfix
+            postfix *= nums[i]
+        return res</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -496,6 +893,11 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
@@ -558,6 +960,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -569,9 +974,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -908,15 +1310,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5244417-A88C-B64D-8BD7-938B8FE8E901}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.83203125" customWidth="1"/>
     <col min="2" max="2" width="21.1640625" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="52.6640625" customWidth="1"/>
+    <col min="4" max="4" width="70.1640625" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
-    <col min="6" max="6" width="124.5" customWidth="1"/>
+    <col min="6" max="6" width="74" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1000,19 +1402,19 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="270" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>25</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -1020,11 +1422,11 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="377" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="13"/>
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="14"/>
       <c r="F6" s="8" t="s">
         <v>27</v>
       </c>
@@ -1049,120 +1451,199 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="204" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="224" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="221" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:6" ht="216" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="180" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="216" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="C10" s="12" t="s">
         <v>49</v>
       </c>
+      <c r="D10" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="F10" s="9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="180" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="198" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>52</v>
+      <c r="B11" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="1"/>
+      <c r="F11" s="13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="221" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="198" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="221" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:6" ht="180" x14ac:dyDescent="0.2">
+      <c r="A13" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="B13" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="5" t="s">
+    </row>
+    <row r="14" spans="1:6" ht="306" x14ac:dyDescent="0.2">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="144" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>63</v>
+      <c r="C16" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="5" customFormat="1" ht="409" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="12" customFormat="1" ht="377" x14ac:dyDescent="0.2">
+      <c r="A18" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="10">
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="B5:B6"/>
@@ -1174,7 +1655,127 @@
     <hyperlink ref="C3" r:id="rId2" xr:uid="{F59E98AA-F1F4-CE41-8F09-82813F1458E9}"/>
     <hyperlink ref="C5" r:id="rId3" xr:uid="{D9FAE911-9873-7840-9F00-39CD70A8E307}"/>
     <hyperlink ref="C7" r:id="rId4" xr:uid="{6617B5C6-0D6E-354C-8095-CD42A8A64706}"/>
-    <hyperlink ref="C8" r:id="rId5" xr:uid="{3F41C5F7-3CCC-4147-AD6E-90DCCB1FB881}"/>
+    <hyperlink ref="C13" r:id="rId5" xr:uid="{34E7F67E-25C2-D744-A819-E01C48332EC7}"/>
+    <hyperlink ref="C16" r:id="rId6" xr:uid="{7ABEB903-6282-9042-AA34-382D8CEC2F54}"/>
+    <hyperlink ref="C18" r:id="rId7" xr:uid="{E13C547E-C915-524E-A947-C927F2DFD37A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFDE5591-DABA-0745-9FCF-F7D90F931FA1}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.5" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" customWidth="1"/>
+    <col min="3" max="3" width="31.83203125" customWidth="1"/>
+    <col min="4" max="4" width="43.83203125" customWidth="1"/>
+    <col min="5" max="5" width="38.6640625" customWidth="1"/>
+    <col min="6" max="6" width="72.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="238" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="12" customFormat="1" ht="306" x14ac:dyDescent="0.2">
+      <c r="A3" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="12" customFormat="1" ht="394" x14ac:dyDescent="0.2">
+      <c r="A4" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="12" customFormat="1" ht="288" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D6" s="12"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{F57987C3-D113-9440-9036-D1C520C7A8C8}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{39AA1842-A478-A549-983B-5B656E568501}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{895007EB-0F5B-4540-8C82-50735A969627}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{90920D12-CD65-BE47-9FEC-E93A23C3E772}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>